<commit_message>
fix(padron): explicar el periodo que Excel convirtio en fecha
Las columnas de periodo que el club agrega a mano no heredan el formato de texto. Un 092026 escrito ahi llega como 92026 y ya se entendia; un 9/2026 lo convierte Excel en fecha y llegaba como un numero de cinco cifras sin sentido, con un mensaje que no ayudaba a encontrar el error. Ahora el mensaje dice que Excel lo guardo como fecha. La hoja de instrucciones lo aclara.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/06-pruebas/PADRON-PRUEBA-v2.xlsx
+++ b/docs/06-pruebas/PADRON-PRUEBA-v2.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="188">
   <si>
     <t>Como completar el padron</t>
   </si>
@@ -129,6 +129,15 @@
     <t>Agregar una sola de las dos columnas hace que se rechace todo el archivo.</t>
   </si>
   <si>
+    <t>En esas columnas nuevas Excel se come el cero de adelante y deja 92026 en vez de</t>
+  </si>
+  <si>
+    <t>092026. No es problema: el sistema lo entiende igual. Lo que si se rechaza es</t>
+  </si>
+  <si>
+    <t>escribir el mes con barra, como 9/2026, porque Excel lo convierte en una fecha.</t>
+  </si>
+  <si>
     <t>Cuando esta listo</t>
   </si>
   <si>
@@ -423,6 +432,12 @@
     <t>Ortega, Olivia</t>
   </si>
   <si>
+    <t>45000003</t>
+  </si>
+  <si>
+    <t>Parcial, Sofia</t>
+  </si>
+  <si>
     <t>42916483</t>
   </si>
   <si>
@@ -447,6 +462,18 @@
     <t>Ponce, Lorena</t>
   </si>
   <si>
+    <t>45000002</t>
+  </si>
+  <si>
+    <t>PostCorte, Mateo</t>
+  </si>
+  <si>
+    <t>45000001</t>
+  </si>
+  <si>
+    <t>PreCorte, Lucia</t>
+  </si>
+  <si>
     <t>39481562</t>
   </si>
   <si>
@@ -487,6 +514,12 @@
   </si>
   <si>
     <t>Serrano, Noelia</t>
+  </si>
+  <si>
+    <t>45000004</t>
+  </si>
+  <si>
+    <t>SinPagos, Tomas</t>
   </si>
   <si>
     <t>39682714</t>
@@ -897,7 +930,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:A60"/>
+  <dimension ref="A1:A64"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="true" style="0"/>
@@ -1089,23 +1122,38 @@
       </c>
     </row>
     <row r="56" spans="1:1">
-      <c r="A56" s="2" t="s">
+      <c r="A56" t="s">
         <v>37</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="58" spans="1:1">
       <c r="A58" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1">
-      <c r="A59" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="60" spans="1:1">
-      <c r="A60" t="s">
+      <c r="A60" s="2" t="s">
         <v>40</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1">
+      <c r="A64" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1120,68 +1168,68 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:P61"/>
+  <dimension ref="A1:P66"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="G1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="I1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="K1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="L1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="M1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="N1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="O1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="P1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:16">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E2" s="1"/>
       <c r="G2" s="1"/>
@@ -1192,13 +1240,13 @@
     </row>
     <row r="3" spans="1:16">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B3" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E3" s="1"/>
       <c r="G3" s="1"/>
@@ -1209,13 +1257,13 @@
     </row>
     <row r="4" spans="1:16">
       <c r="A4" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E4" s="1"/>
       <c r="G4" s="1"/>
@@ -1226,13 +1274,13 @@
     </row>
     <row r="5" spans="1:16">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E5" s="1"/>
       <c r="G5" s="1"/>
@@ -1243,13 +1291,13 @@
     </row>
     <row r="6" spans="1:16">
       <c r="A6" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B6" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C6" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E6" s="1"/>
       <c r="G6" s="1"/>
@@ -1260,13 +1308,13 @@
     </row>
     <row r="7" spans="1:16">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C7" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E7" s="1"/>
       <c r="G7" s="1"/>
@@ -1277,13 +1325,13 @@
     </row>
     <row r="8" spans="1:16">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C8" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E8" s="1"/>
       <c r="G8" s="1"/>
@@ -1294,13 +1342,13 @@
     </row>
     <row r="9" spans="1:16">
       <c r="A9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B9" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E9" s="1"/>
       <c r="G9" s="1"/>
@@ -1311,13 +1359,13 @@
     </row>
     <row r="10" spans="1:16">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B10" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C10" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E10" s="1"/>
       <c r="G10" s="1"/>
@@ -1328,13 +1376,13 @@
     </row>
     <row r="11" spans="1:16">
       <c r="A11" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B11" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E11" s="1"/>
       <c r="G11" s="1"/>
@@ -1345,13 +1393,13 @@
     </row>
     <row r="12" spans="1:16">
       <c r="A12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B12" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C12" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E12" s="1"/>
       <c r="G12" s="1"/>
@@ -1362,13 +1410,13 @@
     </row>
     <row r="13" spans="1:16">
       <c r="A13" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B13" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C13" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E13" s="1"/>
       <c r="G13" s="1"/>
@@ -1379,13 +1427,13 @@
     </row>
     <row r="14" spans="1:16">
       <c r="A14" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B14" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C14" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E14" s="1"/>
       <c r="G14" s="1"/>
@@ -1396,13 +1444,13 @@
     </row>
     <row r="15" spans="1:16">
       <c r="A15" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B15" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C15" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E15" s="1"/>
       <c r="G15" s="1"/>
@@ -1413,13 +1461,13 @@
     </row>
     <row r="16" spans="1:16">
       <c r="A16" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B16" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C16" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E16" s="1"/>
       <c r="G16" s="1"/>
@@ -1430,13 +1478,13 @@
     </row>
     <row r="17" spans="1:16">
       <c r="A17" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B17" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C17" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E17" s="1"/>
       <c r="G17" s="1"/>
@@ -1447,13 +1495,13 @@
     </row>
     <row r="18" spans="1:16">
       <c r="A18" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B18" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C18" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E18" s="1"/>
       <c r="G18" s="1"/>
@@ -1464,13 +1512,13 @@
     </row>
     <row r="19" spans="1:16">
       <c r="A19" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B19" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C19" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E19" s="1"/>
       <c r="G19" s="1"/>
@@ -1481,13 +1529,13 @@
     </row>
     <row r="20" spans="1:16">
       <c r="A20" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B20" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C20" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E20" s="1"/>
       <c r="G20" s="1"/>
@@ -1498,13 +1546,13 @@
     </row>
     <row r="21" spans="1:16">
       <c r="A21" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B21" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C21" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E21" s="1"/>
       <c r="G21" s="1"/>
@@ -1515,13 +1563,13 @@
     </row>
     <row r="22" spans="1:16">
       <c r="A22" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B22" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C22" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E22" s="1"/>
       <c r="G22" s="1"/>
@@ -1532,13 +1580,13 @@
     </row>
     <row r="23" spans="1:16">
       <c r="A23" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B23" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C23" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E23" s="1"/>
       <c r="G23" s="1"/>
@@ -1549,13 +1597,13 @@
     </row>
     <row r="24" spans="1:16">
       <c r="A24" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B24" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C24" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E24" s="1"/>
       <c r="G24" s="1"/>
@@ -1566,13 +1614,13 @@
     </row>
     <row r="25" spans="1:16">
       <c r="A25" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B25" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C25" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E25" s="1"/>
       <c r="G25" s="1"/>
@@ -1583,13 +1631,13 @@
     </row>
     <row r="26" spans="1:16">
       <c r="A26" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B26" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C26" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E26" s="1"/>
       <c r="G26" s="1"/>
@@ -1600,13 +1648,13 @@
     </row>
     <row r="27" spans="1:16">
       <c r="A27" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B27" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C27" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E27" s="1"/>
       <c r="G27" s="1"/>
@@ -1617,13 +1665,13 @@
     </row>
     <row r="28" spans="1:16">
       <c r="A28" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B28" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C28" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E28" s="1"/>
       <c r="G28" s="1"/>
@@ -1634,13 +1682,13 @@
     </row>
     <row r="29" spans="1:16">
       <c r="A29" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B29" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C29" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E29" s="1"/>
       <c r="G29" s="1"/>
@@ -1651,13 +1699,13 @@
     </row>
     <row r="30" spans="1:16">
       <c r="A30" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B30" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C30" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E30" s="1"/>
       <c r="G30" s="1"/>
@@ -1668,13 +1716,13 @@
     </row>
     <row r="31" spans="1:16">
       <c r="A31" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B31" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C31" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E31" s="1"/>
       <c r="G31" s="1"/>
@@ -1685,13 +1733,13 @@
     </row>
     <row r="32" spans="1:16">
       <c r="A32" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B32" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C32" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E32" s="1"/>
       <c r="G32" s="1"/>
@@ -1702,13 +1750,13 @@
     </row>
     <row r="33" spans="1:16">
       <c r="A33" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B33" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C33" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E33" s="1"/>
       <c r="G33" s="1"/>
@@ -1719,13 +1767,13 @@
     </row>
     <row r="34" spans="1:16">
       <c r="A34" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B34" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C34" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E34" s="1"/>
       <c r="G34" s="1"/>
@@ -1736,13 +1784,13 @@
     </row>
     <row r="35" spans="1:16">
       <c r="A35" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B35" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C35" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E35" s="1"/>
       <c r="G35" s="1"/>
@@ -1753,13 +1801,13 @@
     </row>
     <row r="36" spans="1:16">
       <c r="A36" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B36" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C36" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E36" s="1"/>
       <c r="G36" s="1"/>
@@ -1770,13 +1818,13 @@
     </row>
     <row r="37" spans="1:16">
       <c r="A37" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B37" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C37" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E37" s="1"/>
       <c r="G37" s="1"/>
@@ -1787,13 +1835,13 @@
     </row>
     <row r="38" spans="1:16">
       <c r="A38" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B38" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C38" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E38" s="1"/>
       <c r="G38" s="1"/>
@@ -1804,13 +1852,13 @@
     </row>
     <row r="39" spans="1:16">
       <c r="A39" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B39" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C39" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E39" s="1"/>
       <c r="G39" s="1"/>
@@ -1821,13 +1869,13 @@
     </row>
     <row r="40" spans="1:16">
       <c r="A40" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B40" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C40" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E40" s="1"/>
       <c r="G40" s="1"/>
@@ -1838,13 +1886,13 @@
     </row>
     <row r="41" spans="1:16">
       <c r="A41" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B41" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C41" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E41" s="1"/>
       <c r="G41" s="1"/>
@@ -1855,13 +1903,13 @@
     </row>
     <row r="42" spans="1:16">
       <c r="A42" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B42" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C42" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="E42" s="1"/>
       <c r="G42" s="1"/>
@@ -1872,13 +1920,13 @@
     </row>
     <row r="43" spans="1:16">
       <c r="A43" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B43" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C43" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E43" s="1"/>
       <c r="G43" s="1"/>
@@ -1889,13 +1937,13 @@
     </row>
     <row r="44" spans="1:16">
       <c r="A44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B44" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C44" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E44" s="1"/>
       <c r="G44" s="1"/>
@@ -1906,13 +1954,13 @@
     </row>
     <row r="45" spans="1:16">
       <c r="A45" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B45" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C45" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E45" s="1"/>
       <c r="G45" s="1"/>
@@ -1923,13 +1971,13 @@
     </row>
     <row r="46" spans="1:16">
       <c r="A46" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B46" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C46" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="E46" s="1"/>
       <c r="G46" s="1"/>
@@ -1940,13 +1988,13 @@
     </row>
     <row r="47" spans="1:16">
       <c r="A47" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B47" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C47" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E47" s="1"/>
       <c r="G47" s="1"/>
@@ -1957,13 +2005,13 @@
     </row>
     <row r="48" spans="1:16">
       <c r="A48" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B48" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C48" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E48" s="1"/>
       <c r="G48" s="1"/>
@@ -1974,13 +2022,13 @@
     </row>
     <row r="49" spans="1:16">
       <c r="A49" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B49" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C49" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E49" s="1"/>
       <c r="G49" s="1"/>
@@ -1991,13 +2039,13 @@
     </row>
     <row r="50" spans="1:16">
       <c r="A50" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B50" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C50" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E50" s="1"/>
       <c r="G50" s="1"/>
@@ -2008,13 +2056,13 @@
     </row>
     <row r="51" spans="1:16">
       <c r="A51" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B51" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C51" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E51" s="1"/>
       <c r="G51" s="1"/>
@@ -2025,13 +2073,13 @@
     </row>
     <row r="52" spans="1:16">
       <c r="A52" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B52" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C52" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="E52" s="1"/>
       <c r="G52" s="1"/>
@@ -2042,13 +2090,13 @@
     </row>
     <row r="53" spans="1:16">
       <c r="A53" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B53" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C53" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E53" s="1"/>
       <c r="G53" s="1"/>
@@ -2059,13 +2107,13 @@
     </row>
     <row r="54" spans="1:16">
       <c r="A54" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B54" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C54" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E54" s="1"/>
       <c r="G54" s="1"/>
@@ -2076,13 +2124,13 @@
     </row>
     <row r="55" spans="1:16">
       <c r="A55" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B55" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C55" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E55" s="1"/>
       <c r="G55" s="1"/>
@@ -2093,13 +2141,13 @@
     </row>
     <row r="56" spans="1:16">
       <c r="A56" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B56" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C56" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E56" s="1"/>
       <c r="G56" s="1"/>
@@ -2110,13 +2158,13 @@
     </row>
     <row r="57" spans="1:16">
       <c r="A57" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B57" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C57" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E57" s="1"/>
       <c r="G57" s="1"/>
@@ -2127,13 +2175,13 @@
     </row>
     <row r="58" spans="1:16">
       <c r="A58" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B58" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C58" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E58" s="1"/>
       <c r="G58" s="1"/>
@@ -2144,13 +2192,13 @@
     </row>
     <row r="59" spans="1:16">
       <c r="A59" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B59" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C59" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="E59" s="1"/>
       <c r="G59" s="1"/>
@@ -2161,13 +2209,13 @@
     </row>
     <row r="60" spans="1:16">
       <c r="A60" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B60" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C60" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E60" s="1"/>
       <c r="G60" s="1"/>
@@ -2178,13 +2226,13 @@
     </row>
     <row r="61" spans="1:16">
       <c r="A61" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B61" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C61" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E61" s="1"/>
       <c r="G61" s="1"/>
@@ -2193,6 +2241,91 @@
       <c r="M61" s="1"/>
       <c r="O61" s="1"/>
     </row>
+    <row r="62" spans="1:16">
+      <c r="A62" t="s">
+        <v>178</v>
+      </c>
+      <c r="B62" t="s">
+        <v>179</v>
+      </c>
+      <c r="C62" t="s">
+        <v>67</v>
+      </c>
+      <c r="E62" s="1"/>
+      <c r="G62" s="1"/>
+      <c r="I62" s="1"/>
+      <c r="K62" s="1"/>
+      <c r="M62" s="1"/>
+      <c r="O62" s="1"/>
+    </row>
+    <row r="63" spans="1:16">
+      <c r="A63" t="s">
+        <v>180</v>
+      </c>
+      <c r="B63" t="s">
+        <v>181</v>
+      </c>
+      <c r="C63" t="s">
+        <v>67</v>
+      </c>
+      <c r="E63" s="1"/>
+      <c r="G63" s="1"/>
+      <c r="I63" s="1"/>
+      <c r="K63" s="1"/>
+      <c r="M63" s="1"/>
+      <c r="O63" s="1"/>
+    </row>
+    <row r="64" spans="1:16">
+      <c r="A64" t="s">
+        <v>182</v>
+      </c>
+      <c r="B64" t="s">
+        <v>183</v>
+      </c>
+      <c r="C64" t="s">
+        <v>62</v>
+      </c>
+      <c r="E64" s="1"/>
+      <c r="G64" s="1"/>
+      <c r="I64" s="1"/>
+      <c r="K64" s="1"/>
+      <c r="M64" s="1"/>
+      <c r="O64" s="1"/>
+    </row>
+    <row r="65" spans="1:16">
+      <c r="A65" t="s">
+        <v>184</v>
+      </c>
+      <c r="B65" t="s">
+        <v>185</v>
+      </c>
+      <c r="C65" t="s">
+        <v>67</v>
+      </c>
+      <c r="E65" s="1"/>
+      <c r="G65" s="1"/>
+      <c r="I65" s="1"/>
+      <c r="K65" s="1"/>
+      <c r="M65" s="1"/>
+      <c r="O65" s="1"/>
+    </row>
+    <row r="66" spans="1:16">
+      <c r="A66" t="s">
+        <v>186</v>
+      </c>
+      <c r="B66" t="s">
+        <v>187</v>
+      </c>
+      <c r="C66" t="s">
+        <v>67</v>
+      </c>
+      <c r="E66" s="1"/>
+      <c r="G66" s="1"/>
+      <c r="I66" s="1"/>
+      <c r="K66" s="1"/>
+      <c r="M66" s="1"/>
+      <c r="O66" s="1"/>
+    </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>